<commit_message>
Corrige ano da publicação faltante (2021) e melhora legibilidade da rede
- c4ai_publicacoes_manual.xlsx: preenche o ano (2021) do artigo 'Learning to
  sense from events via semantic variational autoencoder' (PLoS One, AGRIBIO).
- Re-roda todo o pipeline: agora 407 publicações todas com ano; AGRIBIO 55;
  pico 2023=189; HHI 1995; top-3 62,7%. Atualiza RELATORIO.md, .tex e README.
- coword_analysis.py: rótulos dos nós deixam de se sobrepor — layout mais
  espalhado, remoção de componentes minúsculos do desenho e adjustText para
  afastar os rótulos (com fundo branco). Aplica também aos painéis temporais.
- Adiciona adjustText às dependências.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Fvrdaa5i99DsPUToDczGGv
</commit_message>
<xml_diff>
--- a/c4ai_publicacoes.xlsx
+++ b/c4ai_publicacoes.xlsx
@@ -1674,7 +1674,9 @@
           <t>AGRIBIO</t>
         </is>
       </c>
-      <c r="B51" t="inlineStr"/>
+      <c r="B51" t="n">
+        <v>2021</v>
+      </c>
       <c r="C51" t="inlineStr">
         <is>
           <t>Learning to sense from events via semantic variational autoencoder</t>

</xml_diff>